<commit_message>
Remove Aura plan from course action tables
</commit_message>
<xml_diff>
--- a/james-street-interview-course/files/kaiying-action-table.xlsx
+++ b/james-street-interview-course/files/kaiying-action-table.xlsx
@@ -9,14 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="黎凯迎_大厂AIPM路线" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="黎凯迎_加入Aura路线" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21天产出总览" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21天产出总览" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'黎凯迎_大厂AIPM路线'!$A$1:$K$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'黎凯迎_加入Aura路线'!$A$1:$K$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'21天产出总览'!$A$1:$D$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'21天产出总览'!$A$1:$D$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -518,16 +516,8 @@
       </c>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>你的加入Aura路线</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>用于判断和准备是否加入赵仁杰的Aura团队。重点是低风险证明价值、清晰角色定位、用户/商户访谈、商业化验证和合作边界。</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="n"/>
     </row>
     <row r="5" ht="52" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -549,7 +539,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>先学当天PPT/讲稿，再填写对应路线表。每一天至少留下一个可检查输出物；没有输出物，就等于没有完成学习。</t>
+          <t>先学当天PPT/讲稿，再填写大厂AIPM路线表。每一天至少留下一个可检查输出物；没有输出物，就等于没有完成学习。</t>
         </is>
       </c>
     </row>
@@ -1182,7 +1172,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>用Aura或任一AI产品模拟收入、成本、回款、留存。</t>
+          <t>用一个AI产品模拟收入、成本、回款、留存。</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1330,7 +1320,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>你可能走大厂，也可能加入初创团队。</t>
+          <t>你需要聚焦大厂AIPM路线。</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1734,1168 +1724,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00657958"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>学习板块</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>核心问题</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>现实处境</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>今日输入</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>今日处理动作</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>今日输出物</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>能力/业务映射</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
-        <is>
-          <t>资产沉淀</t>
-        </is>
-      </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>验证指标</t>
-        </is>
-      </c>
-      <c r="K1" s="4" t="inlineStr">
-        <is>
-          <t>完成记录/复盘</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="78" customHeight="1">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>样本学习</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>我加入强创始人团队时，如何既不崇拜也不低估？</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>赵仁杰履历强、团队信念强，Aura仍处早期验证。</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>用JAMES样本学习法拆Aura和赵仁杰。</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>分清个人优秀、团队执行、产品证据、商业风险。</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Aura创始人/项目样本拆解卡。</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>创业判断；加入前评估</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>为加入前沟通准备证据表。</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>是否能区分“人强”和“项目确定”。</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3" ht="78" customHeight="1">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>资料资产化</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>我能给Aura带去什么方法资产？</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>你可贡献AI资料处理、用户访谈、复盘和课程化能力。</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>整理Aura现有聊天、用户反馈、活动记录、商户信息。</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>设计输入、分类、标签、输出、复盘流程。</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Aura资料加工SOP。</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>PM/FDE；团队方法沉淀</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>成为你加入后的首个贡献物。</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>团队是否能直接按SOP使用。</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4" ht="78" customHeight="1">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>真实开口</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>我能否替团队获取真实用户和商户一手信息？</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Aura有线上用户和线下dating场景，需要更多真人反馈。</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>选3类对象：用户、未转化用户、合作商户。</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>写三套低摩擦访谈邀约。</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Aura一手访谈邀约模板。</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>用户研究；商户调研</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>形成用户访谈入口。</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>是否能拿到至少3个有效回应。</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5" ht="78" customHeight="1">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>身份背书</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>我以什么身份代表Aura提问才可信？</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>你不是创始人，也不是现有PM，需要定义外部沟通身份。</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>梳理你能代表的价值：AI分析、用户研究、活动优化。</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>写用户版、商户版、团队内部版自我介绍。</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Aura访谈可信度介绍模板。</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>角色定位；外部沟通</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>用于商户/用户访谈。</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>对方是否理解你为什么问。</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6" ht="78" customHeight="1">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>问题漏斗</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Aura应该怎样问出用户真实社交需求？</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>dating用户容易说表面偏好，不一定说真实顾虑。</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>参考JAMES固定问题链。</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>改写成相遇经历、动机、顾虑、付费、线下体验7问。</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Aura用户访谈7问脚本。</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>需求挖掘；产品设计</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>团队用户研究基础表。</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>是否能问出具体行为而非空泛偏好。</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="78" customHeight="1">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>追问能力</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>如何追出年轻人玩社交产品背后的真实心理？</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Aura价值在高质量相遇，不是简单匹配。</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>选3类回答：想认识人、怕尴尬、不愿付费。</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>追问背景、动作、顾虑、替代方案、愿付条件。</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Aura深访追问库。</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>用户洞察；付费意愿</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>沉淀为访谈手册。</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>是否能追出可设计的需求。</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8" ht="78" customHeight="1">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>拒绝处理</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>用户和商户拒绝时，我们学到什么？</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>早期产品会遇到不信任、不愿透露、不愿付费。</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>记录一次用户/商户拒绝。</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>拆拒绝原因：时机、价值、价格、安全、信任。</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Aura拒绝处理SOP。</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>销售/运营复盘</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>降低团队对拒绝的情绪化反应。</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>是否能转成下一版话术或产品改动。</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9" ht="78" customHeight="1">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>商业路径</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Aura到底靠什么机制赚钱？</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>目前ToB来自咖啡馆、酒吧、剧本杀，未来探索ToC。</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>列ToB、ToC、线下活动、会员、AI增值、品牌合作路径。</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>按收入来源、成本、壁垒、风险分类。</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Aura商业路径分类表。</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>商业模式；增长判断</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>为路演/团队讨论提供底稿。</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>是否能说清每条路径的钱从哪来。</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10" ht="78" customHeight="1">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>第一桶金</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Aura的第一笔有效收入说明了什么？</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>上线两周用户增长快，但收入质量要验证。</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>整理最早付费商户/活动收入/用户付费信号。</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>拆起点条件、关键动作、可复制性和不可复制项。</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Aura第一收入条件分析。</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>商业验证；PMF前判断</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>形成早期营收证据。</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>是否能判断这笔收入能否重复。</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="78" customHeight="1">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>销售与说服</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>我能否帮Aura把价值卖给商户和用户？</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>ToB靠商户合作，ToC未来要让用户愿意付费。</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>选择咖啡馆/酒吧/剧本杀和C端用户各一类对象。</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>分别写价值pitch：带客、体验、筛选、安全、复购。</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Aura ToB/ToC销售话术。</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>商业化；用户转化</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>用于外联和产品页文案。</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>是否能让对方知道为什么现在合作/付费。</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12" ht="78" customHeight="1">
-      <c r="A12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>现金流</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Aura每场线下活动到底赚不赚钱？</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>ToB收入不等于利润，线下活动有场地、人力、获客成本。</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>列一场活动的收入、成本、转化、复购、退款风险。</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>建立单场活动现金流表。</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Aura线下活动单元模型。</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>ROI；经营分析</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>成为活动复盘固定模板。</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>是否能算出单场活动盈亏平衡点。</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="78" customHeight="1">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>行业机会</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Aura处在dating、AI、线下体验哪个机会交叉点？</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>产品有国内8000+、海外3000+用户，但定位要更精准。</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>拆AI匹配、线下dating、剧本杀/咖啡馆合作、海外用户。</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>按需求增长、付费意愿、进入门槛、团队优势评分。</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Aura机会地图v1。</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>战略定位；赛道判断</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>用于90天重点选择。</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>是否选出最该验证的1-2个切口。</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14" ht="78" customHeight="1">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>杠杆资源</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>我加入后能帮Aura放大什么？</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>团队已有PM、海外成员和创始人资源，你要找到差异位。</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>盘点AI工具、用户访谈、内容、线下商户、数据看板。</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>标注你能承担的杠杆：AI增长/研究/复盘/FDE。</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>个人加入Aura杠杆清单。</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>角色设计；团队分工</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>用于谈职责。</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>是否避免和现有PM重复。</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="78" customHeight="1">
-      <c r="A15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>谈判准备</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>加入前哪些责权利必须讲清楚？</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>朋友团队更容易因为关系不好意思谈边界。</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>列角色、时间、产出、权益、退出、决策权限。</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>准备和赵仁杰的谈判清单。</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>加入前责权利清单。</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>合作边界；风险控制</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>用于正式沟通。</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>是否覆盖钱、权、责、退出。</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16" ht="78" customHeight="1">
-      <c r="A16" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>价值边界</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>我能接受什么样的创业强度和代价？</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>初创可能高成长，也可能消耗时间和求职窗口。</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>写成长、收入、身份、关系、健康、学业的底线。</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>用底线评估加入Aura。</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>加入Aura价值边界表。</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>职业决策；自我管理</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>避免被热情带跑。</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>是否明确不可接受代价。</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="78" customHeight="1">
-      <c r="A17" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>偏差过滤</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>我们会不会把早期数据误读成确定成功？</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>上线两周数据好，但PMF和商业闭环仍需验证。</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>列Aura最容易产生的5个幸存者偏差。</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>写每个偏差的验证方式。</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Aura不可直接乐观清单。</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>风险识别；科学决策</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>帮助团队降温但不打击士气。</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>是否给出可验证证据要求。</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18" ht="78" customHeight="1">
-      <c r="A18" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>传播钩子</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Aura怎么让人愿意看、愿意来、愿意分享？</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>dating产品需要强内容入口，但不能低俗化。</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>拆JAMES数字、身份、反差、悬念钩子。</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>写10个Aura内容钩子：真实相遇、反差、城市、活动。</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Aura内容钩子库。</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>增长内容；品牌表达</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>用于小红书/视频号/活动页。</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>是否既有吸引力又不损害信任。</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="78" customHeight="1">
-      <c r="A19" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>案例包装</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Aura如何讲出真实用户和商户故事？</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>用户成功故事和商户合作故事会影响转化。</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>选择一个线下活动或假设案例。</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>按背景、冲突、关键动作、结果、金句写成案例。</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Aura用户/商户案例模板。</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>品牌叙事；转化素材</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>用于路演、公众号、作品集。</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>案例是否真实、有冲突、有证据。</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20" ht="78" customHeight="1">
-      <c r="A20" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>真实访谈计划</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>加入前我应该先验证哪些问题？</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>你需要低风险证明自己能贡献价值。</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>列用户、商户、团队成员各3个访谈对象。</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>安排7天内完成至少5次访谈。</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>Aura加入前访谈计划。</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>试合作；用户研究</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>作为加入前试任务。</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>是否拿到足够决策信息。</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="78" customHeight="1">
-      <c r="A21" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>AI加工系统</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>我能否帮Aura把反馈持续变成产品判断？</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>早期团队容易让反馈散落在聊天记录和会议里。</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>设计用户反馈和活动复盘字段。</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>建立标签：动机、顾虑、付费、匹配、线下体验、安全。</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>Aura反馈数据库字段设计。</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>AI资料加工；产品运营</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>成为团队知识库。</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>字段是否能支持每周复盘。</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22" ht="78" customHeight="1">
-      <c r="A22" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>30天试合作</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>如果加入，我第一个月交付什么？</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>需要用低风险试合作证明价值，而不是空谈加入。</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>回顾前20天产物。</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>设计30天试合作：访谈、看板、商户话术、内容钩子、复盘。</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>我的Aura 30天试合作行动书。</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>加入路径；价值证明</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>用于和赵仁杰讨论。</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>是否能明确每周产出和验收标准。</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:K22"/>
-  <dataValidations count="1">
-    <dataValidation sqref="K2:K22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"未开始,进行中,已完成,需复盘"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007B563E"/>

</xml_diff>